<commit_message>
Adding fuel costs to different scenarios
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_base1.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_base1.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02A100AD-9271-4861-9548-F151EAA9BBE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CA70EAC-19E2-4DD3-ACF8-DD358F63669B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Co2" sheetId="1" r:id="rId1"/>
+    <sheet name="fuel_costs" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="14">
   <si>
     <t>commodity</t>
   </si>
@@ -57,12 +58,36 @@
   </si>
   <si>
     <t>~TFM_INS-TS</t>
+  </si>
+  <si>
+    <t>~TFM_INS-TS: attribute=flo_cost</t>
+  </si>
+  <si>
+    <t>pset_co</t>
+  </si>
+  <si>
+    <t>Gas</t>
+  </si>
+  <si>
+    <t>Coal</t>
+  </si>
+  <si>
+    <t>Oil</t>
+  </si>
+  <si>
+    <t>Bioenergy</t>
+  </si>
+  <si>
+    <t>wtf?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -92,8 +117,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -109,6 +135,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>457200</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>44742</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>12926</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4BFBA94E-5250-36E0-1C81-B09A479B780D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6064250" y="2235200"/>
+          <a:ext cx="5683542" cy="4407126"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -451,4 +526,191 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F58E262-BA8D-4A3F-93D6-86C72CCD406A}">
+  <dimension ref="A2:I12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="27.90625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3">
+        <v>2022</v>
+      </c>
+      <c r="D3">
+        <v>2025</v>
+      </c>
+      <c r="E3">
+        <v>2030</v>
+      </c>
+      <c r="F3">
+        <v>2035</v>
+      </c>
+      <c r="G3">
+        <v>2040</v>
+      </c>
+      <c r="H3">
+        <v>2045</v>
+      </c>
+      <c r="I3">
+        <v>2050</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="1">
+        <v>35.145058821884028</v>
+      </c>
+      <c r="D4" s="1">
+        <v>35.145058821884028</v>
+      </c>
+      <c r="E4" s="1">
+        <v>34.442157645446351</v>
+      </c>
+      <c r="F4" s="1">
+        <v>33.75331449253742</v>
+      </c>
+      <c r="G4" s="1">
+        <f>F4+F4*0.03</f>
+        <v>34.765913927313541</v>
+      </c>
+      <c r="H4" s="1">
+        <f t="shared" ref="H4:I4" si="0">G4+G4*0.03</f>
+        <v>35.808891345132949</v>
+      </c>
+      <c r="I4" s="1">
+        <f t="shared" si="0"/>
+        <v>36.88315808548694</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="1">
+        <v>96.367112810707454</v>
+      </c>
+      <c r="D5" s="1">
+        <v>96.367112810707454</v>
+      </c>
+      <c r="E5" s="1">
+        <f>D5+(D5*0.03)</f>
+        <v>99.25812619502868</v>
+      </c>
+      <c r="F5" s="1">
+        <f t="shared" ref="F5:I5" si="1">E5+(E5*0.03)</f>
+        <v>102.23586998087954</v>
+      </c>
+      <c r="G5" s="1">
+        <f t="shared" si="1"/>
+        <v>105.30294608030593</v>
+      </c>
+      <c r="H5" s="1">
+        <f t="shared" si="1"/>
+        <v>108.46203446271511</v>
+      </c>
+      <c r="I5" s="1">
+        <f t="shared" si="1"/>
+        <v>111.71589549659656</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="1">
+        <v>46.470588235294123</v>
+      </c>
+      <c r="D6" s="1">
+        <v>46.470588235294123</v>
+      </c>
+      <c r="E6" s="1">
+        <f>D6+(D6*0.03)</f>
+        <v>47.864705882352943</v>
+      </c>
+      <c r="F6" s="1">
+        <f t="shared" ref="F6:I6" si="2">E6+(E6*0.03)</f>
+        <v>49.300647058823529</v>
+      </c>
+      <c r="G6" s="1">
+        <f t="shared" si="2"/>
+        <v>50.779666470588232</v>
+      </c>
+      <c r="H6" s="1">
+        <f t="shared" si="2"/>
+        <v>52.303056464705882</v>
+      </c>
+      <c r="I6" s="1">
+        <f t="shared" si="2"/>
+        <v>53.872148158647057</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="1">
+        <v>45.792000000000002</v>
+      </c>
+      <c r="D7" s="1">
+        <v>45.792000000000002</v>
+      </c>
+      <c r="E7" s="1">
+        <f>D7-(D7*0.02)</f>
+        <v>44.876159999999999</v>
+      </c>
+      <c r="F7" s="1">
+        <f>E7-(E7*0.02)</f>
+        <v>43.978636799999997</v>
+      </c>
+      <c r="G7" s="1">
+        <f t="shared" ref="G7:I7" si="3">F7-(F7*0.02)</f>
+        <v>43.099064063999997</v>
+      </c>
+      <c r="H7" s="1">
+        <f t="shared" si="3"/>
+        <v>42.237082782719995</v>
+      </c>
+      <c r="I7" s="1">
+        <f>H7+(H7*0.02)</f>
+        <v>43.081824438374397</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="I12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Change fuel prices and CO2 to IEA scenarios
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_base1.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_base1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F69D8FF-788A-429A-A7D7-4871D16578F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A099EDE5-EE06-48E6-8804-633C6187E268}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Co2" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="30">
   <si>
     <t>commodity</t>
   </si>
@@ -79,6 +79,54 @@
   </si>
   <si>
     <t>wtf?</t>
+  </si>
+  <si>
+    <t>1ton2GJ</t>
+  </si>
+  <si>
+    <t>1mmbtu2GJ</t>
+  </si>
+  <si>
+    <t>1barrelcrude2GJ</t>
+  </si>
+  <si>
+    <t>MWh2GJ</t>
+  </si>
+  <si>
+    <t>TWh2GJ</t>
+  </si>
+  <si>
+    <t>conversion coeff</t>
+  </si>
+  <si>
+    <t>Fuel prices 2024</t>
+  </si>
+  <si>
+    <t>$/barrel or $/MMBtu</t>
+  </si>
+  <si>
+    <t>$/GJ</t>
+  </si>
+  <si>
+    <t>$/MWh</t>
+  </si>
+  <si>
+    <t>$/TWh</t>
+  </si>
+  <si>
+    <t>MMBtu2twh</t>
+  </si>
+  <si>
+    <t>barrel2twh</t>
+  </si>
+  <si>
+    <t>GAS</t>
+  </si>
+  <si>
+    <t>tonne2twh</t>
+  </si>
+  <si>
+    <t>Biogas</t>
   </si>
 </sst>
 </file>
@@ -117,9 +165,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -138,6 +188,55 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>590550</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>477255</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>133931</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3E7EE6EA-EAED-F420-217F-E3BA78E2C44F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6076950" y="2447925"/>
+          <a:ext cx="7201905" cy="4163006"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -450,14 +549,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A4:I7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -486,7 +585,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -494,18 +593,18 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
       <c r="B7">
-        <v>8.6999999999999994E-2</v>
+        <v>7.2599999999999998E-2</v>
       </c>
       <c r="C7">
-        <v>8.6999999999999994E-2</v>
+        <v>7.2599999999999998E-2</v>
       </c>
       <c r="D7">
-        <v>8.6999999999999994E-2</v>
+        <v>0.08</v>
       </c>
       <c r="E7">
         <v>8.6999999999999994E-2</v>
@@ -525,23 +624,25 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F58E262-BA8D-4A3F-93D6-86C72CCD406A}">
-  <dimension ref="A2:I12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A2:AH17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -570,7 +671,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -587,7 +688,7 @@
         <v>34.442157645446351</v>
       </c>
       <c r="F4" s="1">
-        <v>33.75331449253742</v>
+        <v>31.050488862052873</v>
       </c>
       <c r="G4" s="1">
         <v>34.428380782388167</v>
@@ -596,10 +697,10 @@
         <v>35.11694839803593</v>
       </c>
       <c r="I4" s="1">
-        <v>35.819287365996651</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+        <v>36.168701311841808</v>
+      </c>
+    </row>
+    <row r="5" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -613,22 +714,22 @@
         <v>96.367112810707454</v>
       </c>
       <c r="E5" s="1">
-        <v>94.439770554493307</v>
+        <v>85</v>
       </c>
       <c r="F5" s="1">
-        <v>92.550975143403434</v>
+        <v>79.158699808795419</v>
       </c>
       <c r="G5" s="1">
-        <v>90.699955640535364</v>
+        <v>75</v>
       </c>
       <c r="H5" s="1">
-        <v>88.885956527724659</v>
+        <v>73</v>
       </c>
       <c r="I5" s="1">
-        <v>87.108237397170171</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+        <v>70.554493307839394</v>
+      </c>
+    </row>
+    <row r="6" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -642,22 +743,22 @@
         <v>46.470588235294123</v>
       </c>
       <c r="E6" s="1">
-        <v>58.830000000000005</v>
+        <v>49</v>
       </c>
       <c r="F6" s="1">
-        <v>53.53</v>
+        <v>52.352941176470587</v>
       </c>
       <c r="G6" s="1">
-        <v>53.53</v>
+        <v>55</v>
       </c>
       <c r="H6" s="1">
-        <v>55.120000000000005</v>
+        <v>58</v>
       </c>
       <c r="I6" s="1">
-        <v>60.419999999999995</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+        <v>62.35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -671,24 +772,164 @@
         <v>45.792000000000002</v>
       </c>
       <c r="E7" s="1">
-        <v>24.96</v>
+        <v>48</v>
       </c>
       <c r="F7" s="1">
-        <v>24.96</v>
+        <v>50</v>
       </c>
       <c r="G7" s="1">
-        <v>23.52</v>
+        <v>52</v>
       </c>
       <c r="H7" s="1">
-        <v>23.759999999999998</v>
+        <v>54</v>
       </c>
       <c r="I7" s="1">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" spans="1:34" x14ac:dyDescent="0.25">
       <c r="I12" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="V13" t="s">
+        <v>14</v>
+      </c>
+      <c r="W13" t="s">
+        <v>15</v>
+      </c>
+      <c r="X13" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>18</v>
+      </c>
+      <c r="AB13" t="s">
+        <v>19</v>
+      </c>
+      <c r="AD13" t="s">
+        <v>20</v>
+      </c>
+      <c r="AE13" t="s">
+        <v>21</v>
+      </c>
+      <c r="AF13" t="s">
+        <v>22</v>
+      </c>
+      <c r="AG13" t="s">
+        <v>23</v>
+      </c>
+      <c r="AH13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="V14">
+        <v>4.1840000000000002</v>
+      </c>
+      <c r="W14">
+        <v>1.0550558526</v>
+      </c>
+      <c r="X14">
+        <v>6.12</v>
+      </c>
+      <c r="Y14">
+        <v>3.6</v>
+      </c>
+      <c r="Z14">
+        <v>3600000</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB14">
+        <v>3412142</v>
+      </c>
+      <c r="AD14" t="s">
+        <v>11</v>
+      </c>
+      <c r="AE14">
+        <v>106</v>
+      </c>
+      <c r="AF14" s="2">
+        <f>AE14/X14</f>
+        <v>17.320261437908496</v>
+      </c>
+      <c r="AG14" s="2">
+        <f>AF14*Y14</f>
+        <v>62.352941176470587</v>
+      </c>
+      <c r="AH14" s="2">
+        <f>AF14*Z14</f>
+        <v>62352941.176470585</v>
+      </c>
+    </row>
+    <row r="15" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AA15" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB15" s="3">
+        <v>588235</v>
+      </c>
+      <c r="AD15" t="s">
+        <v>27</v>
+      </c>
+      <c r="AE15">
+        <v>4</v>
+      </c>
+      <c r="AF15" s="2">
+        <f>AE15/W14</f>
+        <v>3.7912684813251372</v>
+      </c>
+      <c r="AG15" s="2">
+        <f>AF15*Y14</f>
+        <v>13.648566532770493</v>
+      </c>
+      <c r="AH15" s="2">
+        <f>AF15*Z14</f>
+        <v>13648566.532770494</v>
+      </c>
+    </row>
+    <row r="16" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AA16" t="s">
+        <v>28</v>
+      </c>
+      <c r="AB16">
+        <v>150000</v>
+      </c>
+      <c r="AD16" t="s">
+        <v>10</v>
+      </c>
+      <c r="AE16">
+        <v>39</v>
+      </c>
+      <c r="AF16" s="2">
+        <f>AE16/V14</f>
+        <v>9.3212237093690238</v>
+      </c>
+      <c r="AG16" s="2">
+        <f>AF16*Y14</f>
+        <v>33.556405353728486</v>
+      </c>
+      <c r="AH16" s="2">
+        <f>AF16*Z14</f>
+        <v>33556405.353728488</v>
+      </c>
+    </row>
+    <row r="17" spans="30:33" x14ac:dyDescent="0.25">
+      <c r="AD17" t="s">
+        <v>29</v>
+      </c>
+      <c r="AF17">
+        <v>12.72</v>
+      </c>
+      <c r="AG17">
+        <f>AF17*Y14</f>
+        <v>45.792000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding fuel and co2 costs to 2022
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_base1.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_base1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{431CE360-47EF-4B3A-9324-941C3E70588F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3745086D-5551-41CE-8D23-73BBA319588F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Co2" sheetId="1" r:id="rId1"/>
@@ -247,9 +247,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>44742</xdr:colOff>
+      <xdr:colOff>54267</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>12926</xdr:rowOff>
+      <xdr:rowOff>16101</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -548,41 +548,44 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A4:H7"/>
+  <dimension ref="A4:I7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>0</v>
       </c>
       <c r="B5">
+        <v>2022</v>
+      </c>
+      <c r="C5">
         <v>2025</v>
       </c>
-      <c r="C5">
+      <c r="D5">
         <v>2030</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>2035</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>2040</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>2045</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>2050</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -590,18 +593,18 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
       <c r="B7">
+        <v>0.08</v>
+      </c>
+      <c r="C7">
         <v>7.2599999999999998E-2</v>
       </c>
-      <c r="C7">
+      <c r="D7">
         <v>0.08</v>
-      </c>
-      <c r="D7">
-        <v>8.6999999999999994E-2</v>
       </c>
       <c r="E7">
         <v>8.6999999999999994E-2</v>
@@ -612,7 +615,10 @@
       <c r="G7">
         <v>8.6999999999999994E-2</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7">
+        <v>8.6999999999999994E-2</v>
+      </c>
+      <c r="I7" t="s">
         <v>5</v>
       </c>
     </row>
@@ -628,6 +634,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -644,21 +651,24 @@
         <v>8</v>
       </c>
       <c r="C3">
+        <v>2022</v>
+      </c>
+      <c r="D3">
         <v>2025</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>2030</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>2035</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>2040</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>2045</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>2050</v>
       </c>
     </row>
@@ -670,21 +680,25 @@
         <v>9</v>
       </c>
       <c r="C4" s="1">
+        <f>D4*(1+0.01)</f>
+        <v>35.496509410102867</v>
+      </c>
+      <c r="D4" s="1">
         <v>35.145058821884028</v>
       </c>
-      <c r="D4" s="1">
+      <c r="E4" s="1">
         <v>34.442157645446351</v>
       </c>
-      <c r="E4" s="1">
+      <c r="F4" s="1">
         <v>31.050488862052873</v>
       </c>
-      <c r="F4" s="1">
+      <c r="G4" s="1">
         <v>34.428380782388167</v>
       </c>
-      <c r="G4" s="1">
+      <c r="H4" s="1">
         <v>35.11694839803593</v>
       </c>
-      <c r="H4" s="1">
+      <c r="I4" s="1">
         <v>36.168701311841808</v>
       </c>
     </row>
@@ -696,21 +710,25 @@
         <v>10</v>
       </c>
       <c r="C5" s="1">
+        <f t="shared" ref="C5:C7" si="0">D5*(1+0.01)</f>
+        <v>97.330783938814534</v>
+      </c>
+      <c r="D5" s="1">
         <v>96.367112810707454</v>
       </c>
-      <c r="D5" s="1">
+      <c r="E5" s="1">
         <v>85</v>
       </c>
-      <c r="E5" s="1">
+      <c r="F5" s="1">
         <v>79.158699808795419</v>
       </c>
-      <c r="F5" s="1">
+      <c r="G5" s="1">
         <v>75</v>
       </c>
-      <c r="G5" s="1">
+      <c r="H5" s="1">
         <v>73</v>
       </c>
-      <c r="H5" s="1">
+      <c r="I5" s="1">
         <v>70.554493307839394</v>
       </c>
     </row>
@@ -722,21 +740,25 @@
         <v>11</v>
       </c>
       <c r="C6" s="1">
+        <f t="shared" si="0"/>
+        <v>46.935294117647068</v>
+      </c>
+      <c r="D6" s="1">
         <v>46.470588235294123</v>
       </c>
-      <c r="D6" s="1">
+      <c r="E6" s="1">
         <v>49</v>
       </c>
-      <c r="E6" s="1">
+      <c r="F6" s="1">
         <v>52.352941176470587</v>
       </c>
-      <c r="F6" s="1">
+      <c r="G6" s="1">
         <v>55</v>
       </c>
-      <c r="G6" s="1">
+      <c r="H6" s="1">
         <v>58</v>
       </c>
-      <c r="H6" s="1">
+      <c r="I6" s="1">
         <v>62.35</v>
       </c>
     </row>
@@ -748,21 +770,25 @@
         <v>12</v>
       </c>
       <c r="C7" s="1">
+        <f t="shared" si="0"/>
+        <v>46.249920000000003</v>
+      </c>
+      <c r="D7" s="1">
         <v>45.792000000000002</v>
       </c>
-      <c r="D7" s="1">
+      <c r="E7" s="1">
         <v>48</v>
       </c>
-      <c r="E7" s="1">
+      <c r="F7" s="1">
         <v>50</v>
       </c>
-      <c r="F7" s="1">
+      <c r="G7" s="1">
         <v>52</v>
       </c>
-      <c r="G7" s="1">
+      <c r="H7" s="1">
         <v>54</v>
       </c>
-      <c r="H7" s="1">
+      <c r="I7" s="1">
         <v>55</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Prettyfy rest of scenario files
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_base1.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_base1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3745086D-5551-41CE-8D23-73BBA319588F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E5D20C5-5C06-4CE0-A89F-1D1F6DD3E7FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Co2" sheetId="1" r:id="rId1"/>
@@ -37,13 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="30">
-  <si>
-    <t>commodity</t>
-  </si>
-  <si>
-    <t>attribute</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="31">
   <si>
     <t>*</t>
   </si>
@@ -60,9 +54,6 @@
     <t>~TFM_INS-TS</t>
   </si>
   <si>
-    <t>~TFM_INS-TS: attribute=flo_cost</t>
-  </si>
-  <si>
     <t>pset_co</t>
   </si>
   <si>
@@ -78,9 +69,6 @@
     <t>Bioenergy</t>
   </si>
   <si>
-    <t>wtf?</t>
-  </si>
-  <si>
     <t>1ton2GJ</t>
   </si>
   <si>
@@ -127,6 +115,21 @@
   </si>
   <si>
     <t>Biogas</t>
+  </si>
+  <si>
+    <t>TimeSlice</t>
+  </si>
+  <si>
+    <t>LimType</t>
+  </si>
+  <si>
+    <t>Attribute</t>
+  </si>
+  <si>
+    <t>Commodity</t>
+  </si>
+  <si>
+    <t>flo_cost</t>
   </si>
 </sst>
 </file>
@@ -136,7 +139,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -144,16 +147,53 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="186"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color indexed="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="43"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="44"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -161,18 +201,36 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 3" xfId="1" xr:uid="{626A6453-D0F9-4A36-ADC9-AF3AE4EFA4C4}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -191,16 +249,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>590550</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>161925</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>477255</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>133931</xdr:rowOff>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>191505</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>95831</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -223,7 +281,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6076950" y="2447925"/>
+          <a:off x="9448800" y="704850"/>
           <a:ext cx="7201905" cy="4163006"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -246,8 +304,8 @@
       <xdr:rowOff>25400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>54267</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>387642</xdr:colOff>
       <xdr:row>36</xdr:row>
       <xdr:rowOff>16101</xdr:rowOff>
     </xdr:to>
@@ -548,78 +606,90 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A4:I7"/>
+  <dimension ref="B6:L9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+    </row>
+    <row r="7" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="7">
+        <v>2022</v>
+      </c>
+      <c r="F7" s="7">
+        <v>2025</v>
+      </c>
+      <c r="G7" s="7">
+        <v>2030</v>
+      </c>
+      <c r="H7" s="7">
+        <v>2035</v>
+      </c>
+      <c r="I7" s="7">
+        <v>2040</v>
+      </c>
+      <c r="J7" s="7">
+        <v>2045</v>
+      </c>
+      <c r="K7" s="7">
+        <v>2050</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B8" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B5">
-        <v>2022</v>
-      </c>
-      <c r="C5">
-        <v>2025</v>
-      </c>
-      <c r="D5">
-        <v>2030</v>
-      </c>
-      <c r="E5">
-        <v>2035</v>
-      </c>
-      <c r="F5">
-        <v>2040</v>
-      </c>
-      <c r="G5">
-        <v>2045</v>
-      </c>
-      <c r="H5">
-        <v>2050</v>
-      </c>
-      <c r="I5" t="s">
+      <c r="C8" s="8" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
+        <v>3</v>
+      </c>
+      <c r="E9">
+        <v>0.08</v>
+      </c>
+      <c r="F9">
+        <v>7.2599999999999998E-2</v>
+      </c>
+      <c r="G9">
+        <v>0.08</v>
+      </c>
+      <c r="H9">
+        <v>8.6999999999999994E-2</v>
+      </c>
+      <c r="I9">
+        <v>8.6999999999999994E-2</v>
+      </c>
+      <c r="J9">
+        <v>8.6999999999999994E-2</v>
+      </c>
+      <c r="K9">
+        <v>8.6999999999999994E-2</v>
+      </c>
+      <c r="L9" t="s">
         <v>2</v>
-      </c>
-      <c r="B6" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7">
-        <v>0.08</v>
-      </c>
-      <c r="C7">
-        <v>7.2599999999999998E-2</v>
-      </c>
-      <c r="D7">
-        <v>0.08</v>
-      </c>
-      <c r="E7">
-        <v>8.6999999999999994E-2</v>
-      </c>
-      <c r="F7">
-        <v>8.6999999999999994E-2</v>
-      </c>
-      <c r="G7">
-        <v>8.6999999999999994E-2</v>
-      </c>
-      <c r="H7">
-        <v>8.6999999999999994E-2</v>
-      </c>
-      <c r="I7" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -630,209 +700,230 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F58E262-BA8D-4A3F-93D6-86C72CCD406A}">
-  <dimension ref="A2:AG17"/>
+  <dimension ref="B2:AG17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="B2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+    </row>
+    <row r="3" spans="2:33" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" s="7">
+        <v>2022</v>
+      </c>
+      <c r="G3" s="7">
+        <v>2025</v>
+      </c>
+      <c r="H3" s="7">
+        <v>2030</v>
+      </c>
+      <c r="I3" s="7">
+        <v>2035</v>
+      </c>
+      <c r="J3" s="7">
+        <v>2040</v>
+      </c>
+      <c r="K3" s="7">
+        <v>2045</v>
+      </c>
+      <c r="L3" s="7">
+        <v>2050</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" s="1">
+        <f>G4*(1+0.01)</f>
+        <v>35.496509410102867</v>
+      </c>
+      <c r="G4" s="1">
+        <v>35.145058821884028</v>
+      </c>
+      <c r="H4" s="1">
+        <v>34.442157645446351</v>
+      </c>
+      <c r="I4" s="1">
+        <v>31.050488862052873</v>
+      </c>
+      <c r="J4" s="1">
+        <v>34.428380782388167</v>
+      </c>
+      <c r="K4" s="1">
+        <v>35.11694839803593</v>
+      </c>
+      <c r="L4" s="1">
+        <v>36.168701311841808</v>
+      </c>
+      <c r="M4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="E5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="1">
+        <f t="shared" ref="F5:F7" si="0">G5*(1+0.01)</f>
+        <v>97.330783938814534</v>
+      </c>
+      <c r="G5" s="1">
+        <v>96.367112810707454</v>
+      </c>
+      <c r="H5" s="1">
+        <v>85</v>
+      </c>
+      <c r="I5" s="1">
+        <v>79.158699808795419</v>
+      </c>
+      <c r="J5" s="1">
+        <v>75</v>
+      </c>
+      <c r="K5" s="1">
+        <v>73</v>
+      </c>
+      <c r="L5" s="1">
+        <v>70.554493307839394</v>
+      </c>
+      <c r="M5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
         <v>8</v>
       </c>
-      <c r="C3">
-        <v>2022</v>
-      </c>
-      <c r="D3">
-        <v>2025</v>
-      </c>
-      <c r="E3">
-        <v>2030</v>
-      </c>
-      <c r="F3">
-        <v>2035</v>
-      </c>
-      <c r="G3">
-        <v>2040</v>
-      </c>
-      <c r="H3">
-        <v>2045</v>
-      </c>
-      <c r="I3">
-        <v>2050</v>
-      </c>
-    </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="1">
-        <f>D4*(1+0.01)</f>
-        <v>35.496509410102867</v>
-      </c>
-      <c r="D4" s="1">
-        <v>35.145058821884028</v>
-      </c>
-      <c r="E4" s="1">
-        <v>34.442157645446351</v>
-      </c>
-      <c r="F4" s="1">
-        <v>31.050488862052873</v>
-      </c>
-      <c r="G4" s="1">
-        <v>34.428380782388167</v>
-      </c>
-      <c r="H4" s="1">
-        <v>35.11694839803593</v>
-      </c>
-      <c r="I4" s="1">
-        <v>36.168701311841808</v>
-      </c>
-    </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="1">
-        <f t="shared" ref="C5:C7" si="0">D5*(1+0.01)</f>
-        <v>97.330783938814534</v>
-      </c>
-      <c r="D5" s="1">
-        <v>96.367112810707454</v>
-      </c>
-      <c r="E5" s="1">
-        <v>85</v>
-      </c>
-      <c r="F5" s="1">
-        <v>79.158699808795419</v>
-      </c>
-      <c r="G5" s="1">
-        <v>75</v>
-      </c>
-      <c r="H5" s="1">
-        <v>73</v>
-      </c>
-      <c r="I5" s="1">
-        <v>70.554493307839394</v>
-      </c>
-    </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="1">
+      <c r="E6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="1">
         <f t="shared" si="0"/>
         <v>46.935294117647068</v>
       </c>
-      <c r="D6" s="1">
+      <c r="G6" s="1">
         <v>46.470588235294123</v>
       </c>
-      <c r="E6" s="1">
+      <c r="H6" s="1">
         <v>49</v>
       </c>
-      <c r="F6" s="1">
+      <c r="I6" s="1">
         <v>52.352941176470587</v>
       </c>
-      <c r="G6" s="1">
+      <c r="J6" s="1">
         <v>55</v>
       </c>
-      <c r="H6" s="1">
+      <c r="K6" s="1">
         <v>58</v>
       </c>
-      <c r="I6" s="1">
+      <c r="L6" s="1">
         <v>62.35</v>
       </c>
-    </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="1">
+      <c r="M6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" s="1">
         <f t="shared" si="0"/>
         <v>46.249920000000003</v>
       </c>
-      <c r="D7" s="1">
+      <c r="G7" s="1">
         <v>45.792000000000002</v>
       </c>
-      <c r="E7" s="1">
+      <c r="H7" s="1">
         <v>48</v>
       </c>
-      <c r="F7" s="1">
+      <c r="I7" s="1">
         <v>50</v>
       </c>
-      <c r="G7" s="1">
+      <c r="J7" s="1">
         <v>52</v>
       </c>
-      <c r="H7" s="1">
+      <c r="K7" s="1">
         <v>54</v>
       </c>
-      <c r="I7" s="1">
+      <c r="L7" s="1">
         <v>55</v>
       </c>
-    </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="H12" t="s">
+      <c r="M7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="2:33" x14ac:dyDescent="0.25">
+      <c r="U13" t="s">
+        <v>10</v>
+      </c>
+      <c r="V13" t="s">
+        <v>11</v>
+      </c>
+      <c r="W13" t="s">
+        <v>12</v>
+      </c>
+      <c r="X13" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="U13" t="s">
+      <c r="Y13" t="s">
         <v>14</v>
       </c>
-      <c r="V13" t="s">
+      <c r="AA13" t="s">
         <v>15</v>
       </c>
-      <c r="W13" t="s">
+      <c r="AC13" t="s">
         <v>16</v>
       </c>
-      <c r="X13" t="s">
+      <c r="AD13" t="s">
         <v>17</v>
       </c>
-      <c r="Y13" t="s">
+      <c r="AE13" t="s">
         <v>18</v>
       </c>
-      <c r="AA13" t="s">
+      <c r="AF13" t="s">
         <v>19</v>
       </c>
-      <c r="AC13" t="s">
+      <c r="AG13" t="s">
         <v>20</v>
       </c>
-      <c r="AD13" t="s">
-        <v>21</v>
-      </c>
-      <c r="AE13" t="s">
-        <v>22</v>
-      </c>
-      <c r="AF13" t="s">
-        <v>23</v>
-      </c>
-      <c r="AG13" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="2:33" x14ac:dyDescent="0.25">
       <c r="U14">
         <v>4.1840000000000002</v>
       </c>
@@ -849,13 +940,13 @@
         <v>3600000</v>
       </c>
       <c r="Z14" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="AA14">
         <v>3412142</v>
       </c>
       <c r="AC14" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="AD14">
         <v>106</v>
@@ -873,15 +964,15 @@
         <v>62352941.176470585</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:33" x14ac:dyDescent="0.25">
       <c r="Z15" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="AA15" s="3">
         <v>588235</v>
       </c>
       <c r="AC15" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="AD15">
         <v>4</v>
@@ -899,15 +990,15 @@
         <v>13648566.532770494</v>
       </c>
     </row>
-    <row r="16" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:33" x14ac:dyDescent="0.25">
       <c r="Z16" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="AA16">
         <v>150000</v>
       </c>
       <c r="AC16" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="AD16">
         <v>39</v>
@@ -927,7 +1018,7 @@
     </row>
     <row r="17" spans="29:32" x14ac:dyDescent="0.25">
       <c r="AC17" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="AE17">
         <v>12.72</v>

</xml_diff>